<commit_message>
chore(issue-77): promote PR Model v4.1
</commit_message>
<xml_diff>
--- a/Info/input/pr_model.xlsx
+++ b/Info/input/pr_model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AI\Downloads\pr_model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\create-pr-cd\Info\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CA657B-26C0-44D5-BCF0-0A33FD4A272F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{95B9EB34-793F-414C-BD74-0772B11E9F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{089DC7BF-D48F-4FC9-B123-3E33291912E1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{089DC7BF-D48F-4FC9-B123-3E33291912E1}"/>
   </bookViews>
   <sheets>
     <sheet name="TX Line Item (After 21-Apr 26)" sheetId="1" r:id="rId1"/>
@@ -1755,7 +1755,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2038" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1693" uniqueCount="174">
   <si>
     <t>TX Site Survey</t>
   </si>
@@ -2264,18 +2264,6 @@
     <t>Decom - Relo</t>
   </si>
   <si>
-    <t>Jendela TX Migration</t>
-  </si>
-  <si>
-    <t>Jendela Model</t>
-  </si>
-  <si>
-    <t>Phase</t>
-  </si>
-  <si>
-    <t>Starlink Dismantle (Return/MRCF included) &amp; Migration</t>
-  </si>
-  <si>
     <t>Starlink Dismantling with 1 antenna（Cage Top）</t>
   </si>
   <si>
@@ -2288,29 +2276,7 @@
     <t>As-built Document and ATP already included</t>
   </si>
   <si>
-    <t>MW Dismantle &amp; MRCF</t>
-  </si>
-  <si>
-    <t>MW Installation</t>
-  </si>
-  <si>
-    <t>Migration from Starlink to MW. All xD sites MW installation by ZTE.
-All Q0xxxx or S0xxxx under xC Jendela project, MW to be installed by Huawei.</t>
-  </si>
-  <si>
-    <t>New Installation</t>
-  </si>
-  <si>
-    <t>Fiber Installation</t>
-  </si>
-  <si>
-    <t>Patching work with seperate mobilization</t>
-  </si>
-  <si>
-    <t>Trip</t>
-  </si>
-  <si>
-    <t>Applicable only for Fiber OB unless TX SOW is BBU Patching</t>
+    <t>Starlink Dismanle</t>
   </si>
 </sst>
 </file>
@@ -2456,7 +2422,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2613,6 +2579,21 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Accent2" xfId="1" builtinId="33"/>
@@ -2621,13 +2602,7 @@
     <cellStyle name="Normal 4 2 2" xfId="4" xr:uid="{AA962A7B-5706-4E11-9052-78D6BBABB481}"/>
     <cellStyle name="常规 116" xfId="3" xr:uid="{D47286A5-C404-4C5F-8EF4-22DB28E47183}"/>
   </cellStyles>
-  <dxfs count="29">
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="27">
     <dxf>
       <font>
         <b val="0"/>
@@ -7545,72 +7520,55 @@
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
   <slicer name="TSS Model 2" xr10:uid="{E33A02A9-D86D-43D1-9039-09161BF92214}" cache="Slicer_TSS_Model111" caption="TSS Model" columnCount="3" rowHeight="144000"/>
-  <slicer name="TI Model 4" xr10:uid="{B4327E0F-182D-45E7-B3D4-958A4D12DC15}" cache="Slicer_TI_Model111" caption="TI Model" columnCount="3" rowHeight="144000"/>
+  <slicer name="TI Model 4" xr10:uid="{B4327E0F-182D-45E7-B3D4-958A4D12DC15}" cache="Slicer_TI_Model111" caption="TI Model" startItem="3" columnCount="3" rowHeight="144000"/>
   <slicer name="Add PR Line Item Model" xr10:uid="{E8947F4E-693E-4B65-9D40-E966E635AD8E}" cache="Slicer_Add_PR_Line_Item_Model" caption="Add PR Line Item Model" rowHeight="234950"/>
 </slicers>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63BE9434-AFC4-4CB4-9E45-994979C6D48E}" name="Table1169" displayName="Table1169" ref="A7:H36" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63BE9434-AFC4-4CB4-9E45-994979C6D48E}" name="Table1169" displayName="Table1169" ref="A7:H36" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A7:H36" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{EC9F81E5-C261-4F84-913A-A8762B1312C9}" name="TSS Model" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{3082E680-9603-4B33-86DF-E70FD7ED2C99}" name="Code" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{A37CA3C1-D74F-485F-BCB7-8DC91B63E87A}" name="Description" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{730F4A6B-FF0F-484F-B58A-7BBE10ACEEFB}" name="Unit" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{8636914A-C6C2-42D8-8FFE-709BAC9BE095}" name="Quantity" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{B76A66B7-2F75-4DA1-87D2-4C4B0C210C18}" name="Rules" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{76A1B753-6759-40D3-985F-AF1ACE921915}" name="Remarks" dataDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{22926371-3F86-47A5-AAC0-948E5FF8B53A}" name="Remarks2" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{EC9F81E5-C261-4F84-913A-A8762B1312C9}" name="TSS Model" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{3082E680-9603-4B33-86DF-E70FD7ED2C99}" name="Code" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{A37CA3C1-D74F-485F-BCB7-8DC91B63E87A}" name="Description" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{730F4A6B-FF0F-484F-B58A-7BBE10ACEEFB}" name="Unit" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{8636914A-C6C2-42D8-8FFE-709BAC9BE095}" name="Quantity" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{B76A66B7-2F75-4DA1-87D2-4C4B0C210C18}" name="Rules" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{76A1B753-6759-40D3-985F-AF1ACE921915}" name="Remarks" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{22926371-3F86-47A5-AAC0-948E5FF8B53A}" name="Remarks2" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E134095E-3A51-4411-AA4E-A7309047E07A}" name="Table12714" displayName="Table12714" ref="A39:G391" totalsRowShown="0" dataDxfId="18">
-  <autoFilter ref="A39:G391" xr:uid="{00000000-0009-0000-0100-00000C000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E134095E-3A51-4411-AA4E-A7309047E07A}" name="Table12714" displayName="Table12714" ref="A39:G393" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="A39:G393" xr:uid="{00000000-0009-0000-0100-00000C000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{291468C8-FDC2-4D9B-A444-194B3C6EFF3C}" name="TI Model" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{28F275E1-BFCC-4FF5-9C11-521DB87DE68F}" name="Code" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{6B7D0885-7542-4368-A983-8D5BA7CDD68B}" name="Description" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{6BA7A254-0F46-4E60-9904-80E088865BAC}" name="Unit" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{52575437-1240-4117-849D-D4A2CDB3A6B3}" name="Quantity" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{DD56CF5C-CA1B-42E1-8AD5-8AC6C2E320C1}" name="Rules" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{F0C4064A-B968-42EE-B9E0-EF2B0CBF1C01}" name="Remarks" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{291468C8-FDC2-4D9B-A444-194B3C6EFF3C}" name="TI Model" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{28F275E1-BFCC-4FF5-9C11-521DB87DE68F}" name="Code" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{6B7D0885-7542-4368-A983-8D5BA7CDD68B}" name="Description" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{6BA7A254-0F46-4E60-9904-80E088865BAC}" name="Unit" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{52575437-1240-4117-849D-D4A2CDB3A6B3}" name="Quantity" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{DD56CF5C-CA1B-42E1-8AD5-8AC6C2E320C1}" name="Rules" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{F0C4064A-B968-42EE-B9E0-EF2B0CBF1C01}" name="Remarks" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4CD2CA86-7CEE-4CD0-B47C-C641CA0F181E}" name="Table3" displayName="Table3" ref="A394:G399" totalsRowShown="0" headerRowDxfId="10" tableBorderDxfId="9">
-  <autoFilter ref="A394:G399" xr:uid="{C921409B-4D8C-4615-9077-350B6EB96C40}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4CD2CA86-7CEE-4CD0-B47C-C641CA0F181E}" name="Table3" displayName="Table3" ref="A396:G401" totalsRowShown="0" headerRowDxfId="8" tableBorderDxfId="7">
+  <autoFilter ref="A396:G401" xr:uid="{C921409B-4D8C-4615-9077-350B6EB96C40}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{31A7B6B0-1197-4056-BDD3-94A5636411E4}" name="Add PR Line Item Model" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{CE2CF9A6-DD5F-4820-AEFE-953E73E863E2}" name="Code" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{2040AADD-8DE9-4F3D-A4BA-363DE5796B06}" name="Description" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{EA415442-6911-4DFE-9C10-B3D349AE27D4}" name="Unit" dataDxfId="5" dataCellStyle="常规 116"/>
-    <tableColumn id="5" xr3:uid="{B4571B37-35C9-408F-A519-45BF32359BAE}" name="Quantity" dataDxfId="4" dataCellStyle="常规 116"/>
-    <tableColumn id="6" xr3:uid="{1B1CCC05-126A-4CDF-A4EE-EFE8F7F19828}" name="Rules" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{CF984CE1-29CF-459A-85E5-C220F87AC4EE}" name="Remarks" dataDxfId="2"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6FE8D8A9-2777-48E3-9B64-F9F2BBA4F91A}" name="Table4" displayName="Table4" ref="A402:H471" totalsRowShown="0">
-  <autoFilter ref="A402:H471" xr:uid="{6FE8D8A9-2777-48E3-9B64-F9F2BBA4F91A}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{3330CE23-3AFE-41D7-B8D6-611EFE913851}" name="Jendela Model"/>
-    <tableColumn id="2" xr3:uid="{3E3B97D8-46C1-4372-A40D-B5F8DBB7A154}" name="Code"/>
-    <tableColumn id="3" xr3:uid="{53E90165-AA05-4EC1-AD62-48E6797BC1F5}" name="Description"/>
-    <tableColumn id="4" xr3:uid="{6F1F1C8E-2E6C-4102-84C3-4B051DC14973}" name="Unit" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{F49F2E89-596F-47D2-985D-392C5220F6CC}" name="Quantity" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{3A7340F3-DE23-4E2D-9566-CE8D16E69ABF}" name="Rules"/>
-    <tableColumn id="7" xr3:uid="{8C07F447-36CD-4AA5-9E86-A150307F366C}" name="Remarks"/>
-    <tableColumn id="8" xr3:uid="{91AC0ADD-EC3E-4BC9-A6A1-4483B2B59D37}" name="Phase"/>
+    <tableColumn id="1" xr3:uid="{31A7B6B0-1197-4056-BDD3-94A5636411E4}" name="Add PR Line Item Model" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{CE2CF9A6-DD5F-4820-AEFE-953E73E863E2}" name="Code" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{2040AADD-8DE9-4F3D-A4BA-363DE5796B06}" name="Description" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{EA415442-6911-4DFE-9C10-B3D349AE27D4}" name="Unit" dataDxfId="3" dataCellStyle="常规 116"/>
+    <tableColumn id="5" xr3:uid="{B4571B37-35C9-408F-A519-45BF32359BAE}" name="Quantity" dataDxfId="2" dataCellStyle="常规 116"/>
+    <tableColumn id="6" xr3:uid="{1B1CCC05-126A-4CDF-A4EE-EFE8F7F19828}" name="Rules" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{CF984CE1-29CF-459A-85E5-C220F87AC4EE}" name="Remarks" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7877,7 +7835,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:H471"/>
+  <dimension ref="A1:H402"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.140625" customWidth="1"/>
@@ -16225,78 +16183,78 @@
       </c>
       <c r="G391" s="21"/>
     </row>
+    <row r="392" spans="1:7">
+      <c r="A392" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B392" s="54">
+        <v>350000597850</v>
+      </c>
+      <c r="C392" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="D392" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E392" s="57">
+        <v>1</v>
+      </c>
+      <c r="F392" s="58" t="s">
+        <v>12</v>
+      </c>
+      <c r="G392" s="21" t="s">
+        <v>170</v>
+      </c>
+    </row>
     <row r="393" spans="1:7">
-      <c r="A393" s="7" t="s">
+      <c r="A393" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B393" s="54">
+        <v>350000597852</v>
+      </c>
+      <c r="C393" s="55" t="s">
+        <v>171</v>
+      </c>
+      <c r="D393" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E393" s="57">
+        <v>1</v>
+      </c>
+      <c r="F393" s="58" t="s">
+        <v>12</v>
+      </c>
+      <c r="G393" s="21" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="395" spans="1:7">
+      <c r="A395" s="7" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="394" spans="1:7">
-      <c r="A394" s="43" t="s">
+    <row r="396" spans="1:7">
+      <c r="A396" s="43" t="s">
         <v>158</v>
       </c>
-      <c r="B394" s="44" t="s">
+      <c r="B396" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="C394" s="44" t="s">
+      <c r="C396" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="D394" s="45" t="s">
+      <c r="D396" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E394" s="44" t="s">
+      <c r="E396" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="F394" s="44" t="s">
+      <c r="F396" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="G394" s="44" t="s">
+      <c r="G396" s="44" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="395" spans="1:7">
-      <c r="A395" s="46" t="s">
-        <v>159</v>
-      </c>
-      <c r="B395" s="47">
-        <v>350001000403</v>
-      </c>
-      <c r="C395" s="46" t="s">
-        <v>160</v>
-      </c>
-      <c r="D395" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="E395" s="49">
-        <v>1</v>
-      </c>
-      <c r="F395" s="50" t="s">
-        <v>77</v>
-      </c>
-      <c r="G395" s="51" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="396" spans="1:7">
-      <c r="A396" s="46" t="s">
-        <v>159</v>
-      </c>
-      <c r="B396" s="47">
-        <v>350001042321</v>
-      </c>
-      <c r="C396" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D396" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="E396" s="49">
-        <v>1</v>
-      </c>
-      <c r="F396" s="50" t="s">
-        <v>77</v>
-      </c>
-      <c r="G396" s="51" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="397" spans="1:7">
@@ -16304,10 +16262,10 @@
         <v>159</v>
       </c>
       <c r="B397" s="47">
-        <v>350001042322</v>
+        <v>350001000403</v>
       </c>
       <c r="C397" s="46" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D397" s="48" t="s">
         <v>19</v>
@@ -16318,19 +16276,19 @@
       <c r="F397" s="50" t="s">
         <v>77</v>
       </c>
-      <c r="G397" s="50" t="s">
-        <v>164</v>
+      <c r="G397" s="51" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="398" spans="1:7">
       <c r="A398" s="46" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B398" s="47">
-        <v>350000592793</v>
+        <v>350001042321</v>
       </c>
       <c r="C398" s="46" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D398" s="48" t="s">
         <v>19</v>
@@ -16339,1675 +16297,99 @@
         <v>1</v>
       </c>
       <c r="F398" s="50" t="s">
-        <v>27</v>
-      </c>
-      <c r="G398" s="50"/>
+        <v>77</v>
+      </c>
+      <c r="G398" s="51" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="399" spans="1:7">
       <c r="A399" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="B399" s="47">
+        <v>350001042322</v>
+      </c>
+      <c r="C399" s="46" t="s">
+        <v>163</v>
+      </c>
+      <c r="D399" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="E399" s="49">
+        <v>1</v>
+      </c>
+      <c r="F399" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="G399" s="50" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="400" spans="1:7">
+      <c r="A400" s="46" t="s">
         <v>165</v>
       </c>
-      <c r="B399" s="47">
+      <c r="B400" s="47">
+        <v>350000592793</v>
+      </c>
+      <c r="C400" s="46" t="s">
+        <v>166</v>
+      </c>
+      <c r="D400" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="E400" s="49">
+        <v>1</v>
+      </c>
+      <c r="F400" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="G400" s="50"/>
+    </row>
+    <row r="401" spans="1:7">
+      <c r="A401" s="46" t="s">
+        <v>165</v>
+      </c>
+      <c r="B401" s="47">
         <v>350000592794</v>
       </c>
-      <c r="C399" s="46" t="s">
+      <c r="C401" s="46" t="s">
         <v>167</v>
       </c>
-      <c r="D399" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="E399" s="49">
-        <v>1</v>
-      </c>
-      <c r="F399" s="50" t="s">
+      <c r="D401" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="E401" s="49">
+        <v>1</v>
+      </c>
+      <c r="F401" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="G399" s="50"/>
-    </row>
-    <row r="400" spans="1:7">
-      <c r="A400" s="52"/>
-      <c r="B400" s="16"/>
-      <c r="C400" s="9"/>
-      <c r="D400" s="12"/>
-      <c r="E400" s="24"/>
-      <c r="F400" s="14"/>
-      <c r="G400" s="53"/>
-    </row>
-    <row r="401" spans="1:8">
-      <c r="A401" s="7" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="402" spans="1:8">
-      <c r="A402" t="s">
-        <v>170</v>
-      </c>
-      <c r="B402" t="s">
-        <v>2</v>
-      </c>
-      <c r="C402" t="s">
-        <v>3</v>
-      </c>
-      <c r="D402" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E402" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="F402" t="s">
-        <v>6</v>
-      </c>
-      <c r="G402" t="s">
-        <v>7</v>
-      </c>
-      <c r="H402" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="403" spans="1:8">
-      <c r="A403" t="s">
-        <v>172</v>
-      </c>
-      <c r="B403">
-        <v>350000597850</v>
-      </c>
-      <c r="C403" t="s">
-        <v>173</v>
-      </c>
-      <c r="D403" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E403" s="5">
-        <v>1</v>
-      </c>
-      <c r="F403" t="s">
-        <v>12</v>
-      </c>
-      <c r="G403" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="404" spans="1:8">
-      <c r="A404" t="s">
-        <v>172</v>
-      </c>
-      <c r="B404">
-        <v>350000597852</v>
-      </c>
-      <c r="C404" t="s">
-        <v>175</v>
-      </c>
-      <c r="D404" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E404" s="5">
-        <v>1</v>
-      </c>
-      <c r="F404" t="s">
-        <v>12</v>
-      </c>
-      <c r="G404" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="405" spans="1:8">
-      <c r="A405" t="s">
-        <v>177</v>
-      </c>
-      <c r="B405">
-        <v>350000589232</v>
-      </c>
-      <c r="C405" t="s">
-        <v>81</v>
-      </c>
-      <c r="D405" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E405" s="5">
-        <v>1</v>
-      </c>
-      <c r="F405" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="406" spans="1:8">
-      <c r="A406" t="s">
-        <v>177</v>
-      </c>
-      <c r="B406">
-        <v>350000589241</v>
-      </c>
-      <c r="C406" t="s">
-        <v>84</v>
-      </c>
-      <c r="D406" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E406" s="5">
-        <v>1</v>
-      </c>
-      <c r="F406" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="407" spans="1:8">
-      <c r="A407" t="s">
-        <v>177</v>
-      </c>
-      <c r="B407">
-        <v>350000589242</v>
-      </c>
-      <c r="C407" t="s">
-        <v>85</v>
-      </c>
-      <c r="D407" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E407" s="5">
-        <v>1</v>
-      </c>
-      <c r="F407" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="408" spans="1:8">
-      <c r="A408" t="s">
-        <v>177</v>
-      </c>
-      <c r="B408">
-        <v>350000589243</v>
-      </c>
-      <c r="C408" t="s">
-        <v>86</v>
-      </c>
-      <c r="D408" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E408" s="5">
-        <v>1</v>
-      </c>
-      <c r="F408" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="409" spans="1:8">
-      <c r="A409" t="s">
-        <v>177</v>
-      </c>
-      <c r="B409">
-        <v>350000589244</v>
-      </c>
-      <c r="C409" t="s">
-        <v>87</v>
-      </c>
-      <c r="D409" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E409" s="5">
-        <v>1</v>
-      </c>
-      <c r="F409" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="410" spans="1:8">
-      <c r="A410" t="s">
-        <v>177</v>
-      </c>
-      <c r="B410">
-        <v>350000589253</v>
-      </c>
-      <c r="C410" t="s">
-        <v>88</v>
-      </c>
-      <c r="D410" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E410" s="5">
-        <v>1</v>
-      </c>
-      <c r="F410" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="411" spans="1:8">
-      <c r="A411" t="s">
-        <v>177</v>
-      </c>
-      <c r="B411">
-        <v>350000589254</v>
-      </c>
-      <c r="C411" t="s">
-        <v>89</v>
-      </c>
-      <c r="D411" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E411" s="5">
-        <v>1</v>
-      </c>
-      <c r="F411" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="412" spans="1:8">
-      <c r="A412" t="s">
-        <v>177</v>
-      </c>
-      <c r="B412">
-        <v>350000589255</v>
-      </c>
-      <c r="C412" t="s">
-        <v>90</v>
-      </c>
-      <c r="D412" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E412" s="5">
-        <v>1</v>
-      </c>
-      <c r="F412" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="413" spans="1:8">
-      <c r="A413" t="s">
-        <v>177</v>
-      </c>
-      <c r="B413">
-        <v>350000589256</v>
-      </c>
-      <c r="C413" t="s">
-        <v>91</v>
-      </c>
-      <c r="D413" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E413" s="5">
-        <v>1</v>
-      </c>
-      <c r="F413" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="414" spans="1:8">
-      <c r="A414" t="s">
-        <v>177</v>
-      </c>
-      <c r="B414">
-        <v>350000589263</v>
-      </c>
-      <c r="C414" t="s">
-        <v>92</v>
-      </c>
-      <c r="D414" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E414" s="5">
-        <v>1</v>
-      </c>
-      <c r="F414" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="415" spans="1:8">
-      <c r="A415" t="s">
-        <v>177</v>
-      </c>
-      <c r="B415">
-        <v>350000589264</v>
-      </c>
-      <c r="C415" t="s">
-        <v>93</v>
-      </c>
-      <c r="D415" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E415" s="5">
-        <v>1</v>
-      </c>
-      <c r="F415" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="416" spans="1:8">
-      <c r="A416" t="s">
-        <v>177</v>
-      </c>
-      <c r="B416">
-        <v>350000589265</v>
-      </c>
-      <c r="C416" t="s">
-        <v>94</v>
-      </c>
-      <c r="D416" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E416" s="5">
-        <v>1</v>
-      </c>
-      <c r="F416" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="417" spans="1:6">
-      <c r="A417" t="s">
-        <v>177</v>
-      </c>
-      <c r="B417">
-        <v>350000589272</v>
-      </c>
-      <c r="C417" t="s">
-        <v>95</v>
-      </c>
-      <c r="D417" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E417" s="5">
-        <v>1</v>
-      </c>
-      <c r="F417" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="418" spans="1:6">
-      <c r="A418" t="s">
-        <v>177</v>
-      </c>
-      <c r="B418">
-        <v>350000589273</v>
-      </c>
-      <c r="C418" t="s">
-        <v>96</v>
-      </c>
-      <c r="D418" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E418" s="5">
-        <v>1</v>
-      </c>
-      <c r="F418" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="419" spans="1:6">
-      <c r="A419" t="s">
-        <v>177</v>
-      </c>
-      <c r="B419">
-        <v>350000589274</v>
-      </c>
-      <c r="C419" t="s">
-        <v>97</v>
-      </c>
-      <c r="D419" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E419" s="5">
-        <v>1</v>
-      </c>
-      <c r="F419" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="420" spans="1:6">
-      <c r="A420" t="s">
-        <v>177</v>
-      </c>
-      <c r="B420">
-        <v>350000589281</v>
-      </c>
-      <c r="C420" t="s">
-        <v>98</v>
-      </c>
-      <c r="D420" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E420" s="5">
-        <v>1</v>
-      </c>
-      <c r="F420" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="421" spans="1:6">
-      <c r="A421" t="s">
-        <v>177</v>
-      </c>
-      <c r="B421">
-        <v>350000589282</v>
-      </c>
-      <c r="C421" t="s">
-        <v>99</v>
-      </c>
-      <c r="D421" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E421" s="5">
-        <v>1</v>
-      </c>
-      <c r="F421" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="422" spans="1:6">
-      <c r="A422" t="s">
-        <v>177</v>
-      </c>
-      <c r="B422">
-        <v>350000589283</v>
-      </c>
-      <c r="C422" t="s">
-        <v>100</v>
-      </c>
-      <c r="D422" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E422" s="5">
-        <v>1</v>
-      </c>
-      <c r="F422" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="423" spans="1:6">
-      <c r="A423" t="s">
-        <v>177</v>
-      </c>
-      <c r="B423">
-        <v>350000589306</v>
-      </c>
-      <c r="C423" t="s">
-        <v>101</v>
-      </c>
-      <c r="D423" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E423" s="5">
-        <v>1</v>
-      </c>
-      <c r="F423" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="424" spans="1:6">
-      <c r="A424" t="s">
-        <v>177</v>
-      </c>
-      <c r="B424">
-        <v>350000589307</v>
-      </c>
-      <c r="C424" t="s">
-        <v>102</v>
-      </c>
-      <c r="D424" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E424" s="5">
-        <v>1</v>
-      </c>
-      <c r="F424" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="425" spans="1:6">
-      <c r="A425" t="s">
-        <v>177</v>
-      </c>
-      <c r="B425">
-        <v>350000589308</v>
-      </c>
-      <c r="C425" t="s">
-        <v>103</v>
-      </c>
-      <c r="D425" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E425" s="5">
-        <v>1</v>
-      </c>
-      <c r="F425" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="426" spans="1:6">
-      <c r="A426" t="s">
-        <v>177</v>
-      </c>
-      <c r="B426">
-        <v>350000589309</v>
-      </c>
-      <c r="C426" t="s">
-        <v>104</v>
-      </c>
-      <c r="D426" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E426" s="5">
-        <v>1</v>
-      </c>
-      <c r="F426" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="427" spans="1:6">
-      <c r="A427" t="s">
-        <v>177</v>
-      </c>
-      <c r="B427">
-        <v>350000589310</v>
-      </c>
-      <c r="C427" t="s">
-        <v>105</v>
-      </c>
-      <c r="D427" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E427" s="5">
-        <v>1</v>
-      </c>
-      <c r="F427" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="428" spans="1:6">
-      <c r="A428" t="s">
-        <v>177</v>
-      </c>
-      <c r="B428">
-        <v>350000589311</v>
-      </c>
-      <c r="C428" t="s">
-        <v>106</v>
-      </c>
-      <c r="D428" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E428" s="5">
-        <v>1</v>
-      </c>
-      <c r="F428" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="429" spans="1:6">
-      <c r="A429" t="s">
-        <v>177</v>
-      </c>
-      <c r="B429">
-        <v>350000589312</v>
-      </c>
-      <c r="C429" t="s">
-        <v>107</v>
-      </c>
-      <c r="D429" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E429" s="5">
-        <v>1</v>
-      </c>
-      <c r="F429" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="430" spans="1:6">
-      <c r="A430" t="s">
-        <v>177</v>
-      </c>
-      <c r="B430">
-        <v>350000589313</v>
-      </c>
-      <c r="C430" t="s">
-        <v>108</v>
-      </c>
-      <c r="D430" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E430" s="5">
-        <v>1</v>
-      </c>
-      <c r="F430" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="431" spans="1:6">
-      <c r="A431" t="s">
-        <v>177</v>
-      </c>
-      <c r="B431">
-        <v>350000589314</v>
-      </c>
-      <c r="C431" t="s">
-        <v>109</v>
-      </c>
-      <c r="D431" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E431" s="5">
-        <v>1</v>
-      </c>
-      <c r="F431" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="432" spans="1:6">
-      <c r="A432" t="s">
-        <v>177</v>
-      </c>
-      <c r="B432">
-        <v>350000589315</v>
-      </c>
-      <c r="C432" t="s">
-        <v>110</v>
-      </c>
-      <c r="D432" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E432" s="5">
-        <v>1</v>
-      </c>
-      <c r="F432" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="433" spans="1:8">
-      <c r="A433" t="s">
-        <v>177</v>
-      </c>
-      <c r="B433">
-        <v>350000589316</v>
-      </c>
-      <c r="C433" t="s">
-        <v>111</v>
-      </c>
-      <c r="D433" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E433" s="5">
-        <v>1</v>
-      </c>
-      <c r="F433" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="434" spans="1:8">
-      <c r="A434" t="s">
-        <v>177</v>
-      </c>
-      <c r="B434">
-        <v>350001095413</v>
-      </c>
-      <c r="C434" t="s">
-        <v>153</v>
-      </c>
-      <c r="D434" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E434" s="5">
-        <v>1</v>
-      </c>
-      <c r="F434" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="435" spans="1:8">
-      <c r="A435" t="s">
-        <v>177</v>
-      </c>
-      <c r="B435">
-        <v>350001095414</v>
-      </c>
-      <c r="C435" t="s">
-        <v>154</v>
-      </c>
-      <c r="D435" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E435" s="5">
-        <v>1</v>
-      </c>
-      <c r="F435" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="436" spans="1:8">
-      <c r="A436" t="s">
-        <v>177</v>
-      </c>
-      <c r="B436">
-        <v>350001095415</v>
-      </c>
-      <c r="C436" t="s">
-        <v>155</v>
-      </c>
-      <c r="D436" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E436" s="5">
-        <v>1</v>
-      </c>
-      <c r="F436" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="437" spans="1:8">
-      <c r="A437" t="s">
-        <v>177</v>
-      </c>
-      <c r="B437">
-        <v>350001095416</v>
-      </c>
-      <c r="C437" t="s">
-        <v>156</v>
-      </c>
-      <c r="D437" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E437" s="5">
-        <v>1</v>
-      </c>
-      <c r="F437" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="438" spans="1:8">
-      <c r="A438" t="s">
-        <v>178</v>
-      </c>
-      <c r="B438">
-        <v>350000214911</v>
-      </c>
-      <c r="C438" t="s">
-        <v>46</v>
-      </c>
-      <c r="D438" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E438" s="5">
-        <v>1</v>
-      </c>
-      <c r="F438" t="s">
-        <v>47</v>
-      </c>
-      <c r="G438" t="s">
-        <v>179</v>
-      </c>
-      <c r="H438" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="439" spans="1:8">
-      <c r="A439" t="s">
-        <v>178</v>
-      </c>
-      <c r="B439">
-        <v>350000214920</v>
-      </c>
-      <c r="C439" t="s">
-        <v>48</v>
-      </c>
-      <c r="D439" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E439" s="5">
-        <v>1</v>
-      </c>
-      <c r="F439" t="s">
-        <v>47</v>
-      </c>
-      <c r="G439" t="s">
-        <v>179</v>
-      </c>
-      <c r="H439" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="440" spans="1:8">
-      <c r="A440" t="s">
-        <v>178</v>
-      </c>
-      <c r="B440">
-        <v>350000214921</v>
-      </c>
-      <c r="C440" t="s">
-        <v>49</v>
-      </c>
-      <c r="D440" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E440" s="5">
-        <v>1</v>
-      </c>
-      <c r="F440" t="s">
-        <v>47</v>
-      </c>
-      <c r="G440" t="s">
-        <v>179</v>
-      </c>
-      <c r="H440" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="441" spans="1:8">
-      <c r="A441" t="s">
-        <v>178</v>
-      </c>
-      <c r="B441">
-        <v>350000214922</v>
-      </c>
-      <c r="C441" t="s">
-        <v>50</v>
-      </c>
-      <c r="D441" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E441" s="5">
-        <v>1</v>
-      </c>
-      <c r="F441" t="s">
-        <v>47</v>
-      </c>
-      <c r="G441" t="s">
-        <v>179</v>
-      </c>
-      <c r="H441" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="442" spans="1:8">
-      <c r="A442" t="s">
-        <v>178</v>
-      </c>
-      <c r="B442">
-        <v>350000214923</v>
-      </c>
-      <c r="C442" t="s">
-        <v>51</v>
-      </c>
-      <c r="D442" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E442" s="5">
-        <v>1</v>
-      </c>
-      <c r="F442" t="s">
-        <v>47</v>
-      </c>
-      <c r="G442" t="s">
-        <v>179</v>
-      </c>
-      <c r="H442" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="443" spans="1:8">
-      <c r="A443" t="s">
-        <v>178</v>
-      </c>
-      <c r="B443">
-        <v>350000475874</v>
-      </c>
-      <c r="C443" t="s">
-        <v>52</v>
-      </c>
-      <c r="D443" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E443" s="5">
-        <v>1</v>
-      </c>
-      <c r="F443" t="s">
-        <v>47</v>
-      </c>
-      <c r="G443" t="s">
-        <v>179</v>
-      </c>
-      <c r="H443" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="444" spans="1:8">
-      <c r="A444" t="s">
-        <v>178</v>
-      </c>
-      <c r="B444">
-        <v>350000475875</v>
-      </c>
-      <c r="C444" t="s">
-        <v>53</v>
-      </c>
-      <c r="D444" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E444" s="5">
-        <v>1</v>
-      </c>
-      <c r="F444" t="s">
-        <v>47</v>
-      </c>
-      <c r="G444" t="s">
-        <v>179</v>
-      </c>
-      <c r="H444" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="445" spans="1:8">
-      <c r="A445" t="s">
-        <v>178</v>
-      </c>
-      <c r="B445">
-        <v>350000475876</v>
-      </c>
-      <c r="C445" t="s">
-        <v>54</v>
-      </c>
-      <c r="D445" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E445" s="5">
-        <v>1</v>
-      </c>
-      <c r="F445" t="s">
-        <v>47</v>
-      </c>
-      <c r="G445" t="s">
-        <v>179</v>
-      </c>
-      <c r="H445" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="446" spans="1:8">
-      <c r="A446" t="s">
-        <v>178</v>
-      </c>
-      <c r="B446">
-        <v>350000475877</v>
-      </c>
-      <c r="C446" t="s">
-        <v>55</v>
-      </c>
-      <c r="D446" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E446" s="5">
-        <v>1</v>
-      </c>
-      <c r="F446" t="s">
-        <v>47</v>
-      </c>
-      <c r="G446" t="s">
-        <v>179</v>
-      </c>
-      <c r="H446" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="447" spans="1:8">
-      <c r="A447" t="s">
-        <v>178</v>
-      </c>
-      <c r="B447">
-        <v>350000214930</v>
-      </c>
-      <c r="C447" t="s">
-        <v>56</v>
-      </c>
-      <c r="D447" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E447" s="5">
-        <v>1</v>
-      </c>
-      <c r="F447" t="s">
-        <v>47</v>
-      </c>
-      <c r="G447" t="s">
-        <v>179</v>
-      </c>
-      <c r="H447" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="448" spans="1:8">
-      <c r="A448" t="s">
-        <v>178</v>
-      </c>
-      <c r="B448">
-        <v>350000214931</v>
-      </c>
-      <c r="C448" t="s">
-        <v>57</v>
-      </c>
-      <c r="D448" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E448" s="5">
-        <v>1</v>
-      </c>
-      <c r="F448" t="s">
-        <v>47</v>
-      </c>
-      <c r="G448" t="s">
-        <v>179</v>
-      </c>
-      <c r="H448" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="449" spans="1:8">
-      <c r="A449" t="s">
-        <v>178</v>
-      </c>
-      <c r="B449">
-        <v>350000214932</v>
-      </c>
-      <c r="C449" t="s">
-        <v>58</v>
-      </c>
-      <c r="D449" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E449" s="5">
-        <v>1</v>
-      </c>
-      <c r="F449" t="s">
-        <v>47</v>
-      </c>
-      <c r="G449" t="s">
-        <v>179</v>
-      </c>
-      <c r="H449" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="450" spans="1:8">
-      <c r="A450" t="s">
-        <v>178</v>
-      </c>
-      <c r="B450">
-        <v>350000214939</v>
-      </c>
-      <c r="C450" t="s">
-        <v>59</v>
-      </c>
-      <c r="D450" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E450" s="5">
-        <v>1</v>
-      </c>
-      <c r="F450" t="s">
-        <v>47</v>
-      </c>
-      <c r="G450" t="s">
-        <v>179</v>
-      </c>
-      <c r="H450" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="451" spans="1:8">
-      <c r="A451" t="s">
-        <v>178</v>
-      </c>
-      <c r="B451">
-        <v>350000214940</v>
-      </c>
-      <c r="C451" t="s">
-        <v>60</v>
-      </c>
-      <c r="D451" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E451" s="5">
-        <v>1</v>
-      </c>
-      <c r="F451" t="s">
-        <v>47</v>
-      </c>
-      <c r="G451" t="s">
-        <v>179</v>
-      </c>
-      <c r="H451" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="452" spans="1:8">
-      <c r="A452" t="s">
-        <v>178</v>
-      </c>
-      <c r="B452">
-        <v>350000214941</v>
-      </c>
-      <c r="C452" t="s">
-        <v>61</v>
-      </c>
-      <c r="D452" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E452" s="5">
-        <v>1</v>
-      </c>
-      <c r="F452" t="s">
-        <v>47</v>
-      </c>
-      <c r="G452" t="s">
-        <v>179</v>
-      </c>
-      <c r="H452" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="453" spans="1:8">
-      <c r="A453" t="s">
-        <v>178</v>
-      </c>
-      <c r="B453">
-        <v>350000298408</v>
-      </c>
-      <c r="C453" t="s">
-        <v>62</v>
-      </c>
-      <c r="D453" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E453" s="5">
-        <v>1</v>
-      </c>
-      <c r="F453" t="s">
-        <v>47</v>
-      </c>
-      <c r="G453" t="s">
-        <v>179</v>
-      </c>
-      <c r="H453" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="454" spans="1:8">
-      <c r="A454" t="s">
-        <v>178</v>
-      </c>
-      <c r="B454">
-        <v>350000298409</v>
-      </c>
-      <c r="C454" t="s">
-        <v>63</v>
-      </c>
-      <c r="D454" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E454" s="5">
-        <v>1</v>
-      </c>
-      <c r="F454" t="s">
-        <v>47</v>
-      </c>
-      <c r="G454" t="s">
-        <v>179</v>
-      </c>
-      <c r="H454" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="455" spans="1:8">
-      <c r="A455" t="s">
-        <v>178</v>
-      </c>
-      <c r="B455">
-        <v>350000298410</v>
-      </c>
-      <c r="C455" t="s">
-        <v>64</v>
-      </c>
-      <c r="D455" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E455" s="5">
-        <v>1</v>
-      </c>
-      <c r="F455" t="s">
-        <v>47</v>
-      </c>
-      <c r="G455" t="s">
-        <v>179</v>
-      </c>
-      <c r="H455" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="456" spans="1:8">
-      <c r="A456" t="s">
-        <v>178</v>
-      </c>
-      <c r="B456">
-        <v>350000212468</v>
-      </c>
-      <c r="C456" t="s">
-        <v>65</v>
-      </c>
-      <c r="D456" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E456" s="5">
-        <v>1</v>
-      </c>
-      <c r="F456" t="s">
-        <v>47</v>
-      </c>
-      <c r="G456" t="s">
-        <v>179</v>
-      </c>
-      <c r="H456" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="457" spans="1:8">
-      <c r="A457" t="s">
-        <v>178</v>
-      </c>
-      <c r="B457">
-        <v>350000212469</v>
-      </c>
-      <c r="C457" t="s">
-        <v>66</v>
-      </c>
-      <c r="D457" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E457" s="5">
-        <v>1</v>
-      </c>
-      <c r="F457" t="s">
-        <v>47</v>
-      </c>
-      <c r="G457" t="s">
-        <v>179</v>
-      </c>
-      <c r="H457" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="458" spans="1:8">
-      <c r="A458" t="s">
-        <v>178</v>
-      </c>
-      <c r="B458">
-        <v>350000212470</v>
-      </c>
-      <c r="C458" t="s">
-        <v>67</v>
-      </c>
-      <c r="D458" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E458" s="5">
-        <v>1</v>
-      </c>
-      <c r="F458" t="s">
-        <v>47</v>
-      </c>
-      <c r="G458" t="s">
-        <v>179</v>
-      </c>
-      <c r="H458" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="459" spans="1:8">
-      <c r="A459" t="s">
-        <v>178</v>
-      </c>
-      <c r="B459">
-        <v>350000212471</v>
-      </c>
-      <c r="C459" t="s">
-        <v>68</v>
-      </c>
-      <c r="D459" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E459" s="5">
-        <v>1</v>
-      </c>
-      <c r="F459" t="s">
-        <v>47</v>
-      </c>
-      <c r="G459" t="s">
-        <v>179</v>
-      </c>
-      <c r="H459" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="460" spans="1:8">
-      <c r="A460" t="s">
-        <v>178</v>
-      </c>
-      <c r="B460">
-        <v>350000212472</v>
-      </c>
-      <c r="C460" t="s">
-        <v>69</v>
-      </c>
-      <c r="D460" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E460" s="5">
-        <v>1</v>
-      </c>
-      <c r="F460" t="s">
-        <v>47</v>
-      </c>
-      <c r="G460" t="s">
-        <v>179</v>
-      </c>
-      <c r="H460" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="461" spans="1:8">
-      <c r="A461" t="s">
-        <v>178</v>
-      </c>
-      <c r="B461">
-        <v>350000212473</v>
-      </c>
-      <c r="C461" t="s">
-        <v>70</v>
-      </c>
-      <c r="D461" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E461" s="5">
-        <v>1</v>
-      </c>
-      <c r="F461" t="s">
-        <v>47</v>
-      </c>
-      <c r="G461" t="s">
-        <v>179</v>
-      </c>
-      <c r="H461" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="462" spans="1:8">
-      <c r="A462" t="s">
-        <v>178</v>
-      </c>
-      <c r="B462">
-        <v>350000358611</v>
-      </c>
-      <c r="C462" t="s">
-        <v>71</v>
-      </c>
-      <c r="D462" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E462" s="5">
-        <v>1</v>
-      </c>
-      <c r="F462" t="s">
-        <v>47</v>
-      </c>
-      <c r="G462" t="s">
-        <v>179</v>
-      </c>
-      <c r="H462" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="463" spans="1:8">
-      <c r="A463" t="s">
-        <v>178</v>
-      </c>
-      <c r="B463">
-        <v>350000212474</v>
-      </c>
-      <c r="C463" t="s">
-        <v>72</v>
-      </c>
-      <c r="D463" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E463" s="5">
-        <v>1</v>
-      </c>
-      <c r="F463" t="s">
-        <v>47</v>
-      </c>
-      <c r="G463" t="s">
-        <v>179</v>
-      </c>
-      <c r="H463" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="464" spans="1:8">
-      <c r="A464" t="s">
-        <v>178</v>
-      </c>
-      <c r="B464">
-        <v>350000212475</v>
-      </c>
-      <c r="C464" t="s">
-        <v>73</v>
-      </c>
-      <c r="D464" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E464" s="5">
-        <v>1</v>
-      </c>
-      <c r="F464" t="s">
-        <v>47</v>
-      </c>
-      <c r="G464" t="s">
-        <v>179</v>
-      </c>
-      <c r="H464" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="465" spans="1:8">
-      <c r="A465" t="s">
-        <v>178</v>
-      </c>
-      <c r="B465">
-        <v>350000212476</v>
-      </c>
-      <c r="C465" t="s">
-        <v>74</v>
-      </c>
-      <c r="D465" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E465" s="5">
-        <v>1</v>
-      </c>
-      <c r="F465" t="s">
-        <v>47</v>
-      </c>
-      <c r="G465" t="s">
-        <v>179</v>
-      </c>
-      <c r="H465" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="466" spans="1:8">
-      <c r="A466" t="s">
-        <v>178</v>
-      </c>
-      <c r="B466">
-        <v>350000589206</v>
-      </c>
-      <c r="C466" t="s">
-        <v>75</v>
-      </c>
-      <c r="D466" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E466" s="5">
-        <v>1</v>
-      </c>
-      <c r="F466" t="s">
-        <v>47</v>
-      </c>
-      <c r="G466" t="s">
-        <v>179</v>
-      </c>
-      <c r="H466" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="467" spans="1:8">
-      <c r="A467" t="s">
-        <v>178</v>
-      </c>
-      <c r="B467">
-        <v>350001095409</v>
-      </c>
-      <c r="C467" t="s">
-        <v>132</v>
-      </c>
-      <c r="D467" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E467" s="5">
-        <v>1</v>
-      </c>
-      <c r="F467" t="s">
-        <v>133</v>
-      </c>
-      <c r="G467" t="s">
-        <v>179</v>
-      </c>
-      <c r="H467" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="468" spans="1:8">
-      <c r="A468" t="s">
-        <v>178</v>
-      </c>
-      <c r="B468">
-        <v>350001095410</v>
-      </c>
-      <c r="C468" t="s">
-        <v>134</v>
-      </c>
-      <c r="D468" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E468" s="5">
-        <v>1</v>
-      </c>
-      <c r="F468" t="s">
-        <v>133</v>
-      </c>
-      <c r="G468" t="s">
-        <v>179</v>
-      </c>
-      <c r="H468" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="469" spans="1:8">
-      <c r="A469" t="s">
-        <v>178</v>
-      </c>
-      <c r="B469">
-        <v>350001095411</v>
-      </c>
-      <c r="C469" t="s">
-        <v>135</v>
-      </c>
-      <c r="D469" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E469" s="5">
-        <v>1</v>
-      </c>
-      <c r="F469" t="s">
-        <v>133</v>
-      </c>
-      <c r="G469" t="s">
-        <v>179</v>
-      </c>
-      <c r="H469" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="470" spans="1:8">
-      <c r="A470" t="s">
-        <v>178</v>
-      </c>
-      <c r="B470">
-        <v>350001095412</v>
-      </c>
-      <c r="C470" t="s">
-        <v>136</v>
-      </c>
-      <c r="D470" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E470" s="5">
-        <v>1</v>
-      </c>
-      <c r="F470" t="s">
-        <v>133</v>
-      </c>
-      <c r="G470" t="s">
-        <v>179</v>
-      </c>
-      <c r="H470" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="471" spans="1:8">
-      <c r="A471" t="s">
-        <v>181</v>
-      </c>
-      <c r="B471">
-        <v>350000499960</v>
-      </c>
-      <c r="C471" t="s">
-        <v>182</v>
-      </c>
-      <c r="D471" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="E471" s="5">
-        <v>1</v>
-      </c>
-      <c r="F471" t="s">
-        <v>12</v>
-      </c>
-      <c r="G471" t="s">
-        <v>184</v>
-      </c>
-      <c r="H471" t="s">
-        <v>180</v>
-      </c>
+      <c r="G401" s="50"/>
+    </row>
+    <row r="402" spans="1:7">
+      <c r="A402" s="52"/>
+      <c r="B402" s="16"/>
+      <c r="C402" s="9"/>
+      <c r="D402" s="12"/>
+      <c r="E402" s="24"/>
+      <c r="F402" s="14"/>
+      <c r="G402" s="53"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="37" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
-  <tableParts count="4">
+  <tableParts count="3">
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
-    <tablePart r:id="rId6"/>
   </tableParts>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{3A4CF648-6AED-40f4-86FF-DC5316D8AED3}">
       <x14:slicerList xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicer r:id="rId7"/>
+        <x14:slicer r:id="rId6"/>
       </x14:slicerList>
     </ext>
   </extLst>

</xml_diff>

<commit_message>
fix(issue-77): redesign Jendela TX migration decision model (#79)
Redesign Jendela TX Migration TI decisions around TX Before Migration and Tx SOW, remove Final Backhaul from decision/blocking, align production PR Model v4.1 and its audit metadata, preserve global no-output/atomic safeguards, and add regression coverage.

Fixes #77
</commit_message>
<xml_diff>
--- a/Info/input/pr_model.xlsx
+++ b/Info/input/pr_model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AI\Downloads\pr_model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\create-pr-cd\Info\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CA657B-26C0-44D5-BCF0-0A33FD4A272F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{95B9EB34-793F-414C-BD74-0772B11E9F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{089DC7BF-D48F-4FC9-B123-3E33291912E1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{089DC7BF-D48F-4FC9-B123-3E33291912E1}"/>
   </bookViews>
   <sheets>
     <sheet name="TX Line Item (After 21-Apr 26)" sheetId="1" r:id="rId1"/>
@@ -1755,7 +1755,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2038" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1693" uniqueCount="174">
   <si>
     <t>TX Site Survey</t>
   </si>
@@ -2264,18 +2264,6 @@
     <t>Decom - Relo</t>
   </si>
   <si>
-    <t>Jendela TX Migration</t>
-  </si>
-  <si>
-    <t>Jendela Model</t>
-  </si>
-  <si>
-    <t>Phase</t>
-  </si>
-  <si>
-    <t>Starlink Dismantle (Return/MRCF included) &amp; Migration</t>
-  </si>
-  <si>
     <t>Starlink Dismantling with 1 antenna（Cage Top）</t>
   </si>
   <si>
@@ -2288,29 +2276,7 @@
     <t>As-built Document and ATP already included</t>
   </si>
   <si>
-    <t>MW Dismantle &amp; MRCF</t>
-  </si>
-  <si>
-    <t>MW Installation</t>
-  </si>
-  <si>
-    <t>Migration from Starlink to MW. All xD sites MW installation by ZTE.
-All Q0xxxx or S0xxxx under xC Jendela project, MW to be installed by Huawei.</t>
-  </si>
-  <si>
-    <t>New Installation</t>
-  </si>
-  <si>
-    <t>Fiber Installation</t>
-  </si>
-  <si>
-    <t>Patching work with seperate mobilization</t>
-  </si>
-  <si>
-    <t>Trip</t>
-  </si>
-  <si>
-    <t>Applicable only for Fiber OB unless TX SOW is BBU Patching</t>
+    <t>Starlink Dismanle</t>
   </si>
 </sst>
 </file>
@@ -2456,7 +2422,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2613,6 +2579,21 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Accent2" xfId="1" builtinId="33"/>
@@ -2621,13 +2602,7 @@
     <cellStyle name="Normal 4 2 2" xfId="4" xr:uid="{AA962A7B-5706-4E11-9052-78D6BBABB481}"/>
     <cellStyle name="常规 116" xfId="3" xr:uid="{D47286A5-C404-4C5F-8EF4-22DB28E47183}"/>
   </cellStyles>
-  <dxfs count="29">
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="27">
     <dxf>
       <font>
         <b val="0"/>
@@ -7545,72 +7520,55 @@
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
   <slicer name="TSS Model 2" xr10:uid="{E33A02A9-D86D-43D1-9039-09161BF92214}" cache="Slicer_TSS_Model111" caption="TSS Model" columnCount="3" rowHeight="144000"/>
-  <slicer name="TI Model 4" xr10:uid="{B4327E0F-182D-45E7-B3D4-958A4D12DC15}" cache="Slicer_TI_Model111" caption="TI Model" columnCount="3" rowHeight="144000"/>
+  <slicer name="TI Model 4" xr10:uid="{B4327E0F-182D-45E7-B3D4-958A4D12DC15}" cache="Slicer_TI_Model111" caption="TI Model" startItem="3" columnCount="3" rowHeight="144000"/>
   <slicer name="Add PR Line Item Model" xr10:uid="{E8947F4E-693E-4B65-9D40-E966E635AD8E}" cache="Slicer_Add_PR_Line_Item_Model" caption="Add PR Line Item Model" rowHeight="234950"/>
 </slicers>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63BE9434-AFC4-4CB4-9E45-994979C6D48E}" name="Table1169" displayName="Table1169" ref="A7:H36" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63BE9434-AFC4-4CB4-9E45-994979C6D48E}" name="Table1169" displayName="Table1169" ref="A7:H36" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A7:H36" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{EC9F81E5-C261-4F84-913A-A8762B1312C9}" name="TSS Model" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{3082E680-9603-4B33-86DF-E70FD7ED2C99}" name="Code" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{A37CA3C1-D74F-485F-BCB7-8DC91B63E87A}" name="Description" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{730F4A6B-FF0F-484F-B58A-7BBE10ACEEFB}" name="Unit" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{8636914A-C6C2-42D8-8FFE-709BAC9BE095}" name="Quantity" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{B76A66B7-2F75-4DA1-87D2-4C4B0C210C18}" name="Rules" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{76A1B753-6759-40D3-985F-AF1ACE921915}" name="Remarks" dataDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{22926371-3F86-47A5-AAC0-948E5FF8B53A}" name="Remarks2" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{EC9F81E5-C261-4F84-913A-A8762B1312C9}" name="TSS Model" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{3082E680-9603-4B33-86DF-E70FD7ED2C99}" name="Code" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{A37CA3C1-D74F-485F-BCB7-8DC91B63E87A}" name="Description" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{730F4A6B-FF0F-484F-B58A-7BBE10ACEEFB}" name="Unit" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{8636914A-C6C2-42D8-8FFE-709BAC9BE095}" name="Quantity" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{B76A66B7-2F75-4DA1-87D2-4C4B0C210C18}" name="Rules" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{76A1B753-6759-40D3-985F-AF1ACE921915}" name="Remarks" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{22926371-3F86-47A5-AAC0-948E5FF8B53A}" name="Remarks2" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E134095E-3A51-4411-AA4E-A7309047E07A}" name="Table12714" displayName="Table12714" ref="A39:G391" totalsRowShown="0" dataDxfId="18">
-  <autoFilter ref="A39:G391" xr:uid="{00000000-0009-0000-0100-00000C000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E134095E-3A51-4411-AA4E-A7309047E07A}" name="Table12714" displayName="Table12714" ref="A39:G393" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="A39:G393" xr:uid="{00000000-0009-0000-0100-00000C000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{291468C8-FDC2-4D9B-A444-194B3C6EFF3C}" name="TI Model" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{28F275E1-BFCC-4FF5-9C11-521DB87DE68F}" name="Code" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{6B7D0885-7542-4368-A983-8D5BA7CDD68B}" name="Description" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{6BA7A254-0F46-4E60-9904-80E088865BAC}" name="Unit" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{52575437-1240-4117-849D-D4A2CDB3A6B3}" name="Quantity" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{DD56CF5C-CA1B-42E1-8AD5-8AC6C2E320C1}" name="Rules" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{F0C4064A-B968-42EE-B9E0-EF2B0CBF1C01}" name="Remarks" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{291468C8-FDC2-4D9B-A444-194B3C6EFF3C}" name="TI Model" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{28F275E1-BFCC-4FF5-9C11-521DB87DE68F}" name="Code" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{6B7D0885-7542-4368-A983-8D5BA7CDD68B}" name="Description" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{6BA7A254-0F46-4E60-9904-80E088865BAC}" name="Unit" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{52575437-1240-4117-849D-D4A2CDB3A6B3}" name="Quantity" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{DD56CF5C-CA1B-42E1-8AD5-8AC6C2E320C1}" name="Rules" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{F0C4064A-B968-42EE-B9E0-EF2B0CBF1C01}" name="Remarks" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4CD2CA86-7CEE-4CD0-B47C-C641CA0F181E}" name="Table3" displayName="Table3" ref="A394:G399" totalsRowShown="0" headerRowDxfId="10" tableBorderDxfId="9">
-  <autoFilter ref="A394:G399" xr:uid="{C921409B-4D8C-4615-9077-350B6EB96C40}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4CD2CA86-7CEE-4CD0-B47C-C641CA0F181E}" name="Table3" displayName="Table3" ref="A396:G401" totalsRowShown="0" headerRowDxfId="8" tableBorderDxfId="7">
+  <autoFilter ref="A396:G401" xr:uid="{C921409B-4D8C-4615-9077-350B6EB96C40}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{31A7B6B0-1197-4056-BDD3-94A5636411E4}" name="Add PR Line Item Model" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{CE2CF9A6-DD5F-4820-AEFE-953E73E863E2}" name="Code" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{2040AADD-8DE9-4F3D-A4BA-363DE5796B06}" name="Description" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{EA415442-6911-4DFE-9C10-B3D349AE27D4}" name="Unit" dataDxfId="5" dataCellStyle="常规 116"/>
-    <tableColumn id="5" xr3:uid="{B4571B37-35C9-408F-A519-45BF32359BAE}" name="Quantity" dataDxfId="4" dataCellStyle="常规 116"/>
-    <tableColumn id="6" xr3:uid="{1B1CCC05-126A-4CDF-A4EE-EFE8F7F19828}" name="Rules" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{CF984CE1-29CF-459A-85E5-C220F87AC4EE}" name="Remarks" dataDxfId="2"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6FE8D8A9-2777-48E3-9B64-F9F2BBA4F91A}" name="Table4" displayName="Table4" ref="A402:H471" totalsRowShown="0">
-  <autoFilter ref="A402:H471" xr:uid="{6FE8D8A9-2777-48E3-9B64-F9F2BBA4F91A}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{3330CE23-3AFE-41D7-B8D6-611EFE913851}" name="Jendela Model"/>
-    <tableColumn id="2" xr3:uid="{3E3B97D8-46C1-4372-A40D-B5F8DBB7A154}" name="Code"/>
-    <tableColumn id="3" xr3:uid="{53E90165-AA05-4EC1-AD62-48E6797BC1F5}" name="Description"/>
-    <tableColumn id="4" xr3:uid="{6F1F1C8E-2E6C-4102-84C3-4B051DC14973}" name="Unit" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{F49F2E89-596F-47D2-985D-392C5220F6CC}" name="Quantity" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{3A7340F3-DE23-4E2D-9566-CE8D16E69ABF}" name="Rules"/>
-    <tableColumn id="7" xr3:uid="{8C07F447-36CD-4AA5-9E86-A150307F366C}" name="Remarks"/>
-    <tableColumn id="8" xr3:uid="{91AC0ADD-EC3E-4BC9-A6A1-4483B2B59D37}" name="Phase"/>
+    <tableColumn id="1" xr3:uid="{31A7B6B0-1197-4056-BDD3-94A5636411E4}" name="Add PR Line Item Model" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{CE2CF9A6-DD5F-4820-AEFE-953E73E863E2}" name="Code" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{2040AADD-8DE9-4F3D-A4BA-363DE5796B06}" name="Description" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{EA415442-6911-4DFE-9C10-B3D349AE27D4}" name="Unit" dataDxfId="3" dataCellStyle="常规 116"/>
+    <tableColumn id="5" xr3:uid="{B4571B37-35C9-408F-A519-45BF32359BAE}" name="Quantity" dataDxfId="2" dataCellStyle="常规 116"/>
+    <tableColumn id="6" xr3:uid="{1B1CCC05-126A-4CDF-A4EE-EFE8F7F19828}" name="Rules" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{CF984CE1-29CF-459A-85E5-C220F87AC4EE}" name="Remarks" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7877,7 +7835,7 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:H471"/>
+  <dimension ref="A1:H402"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.140625" customWidth="1"/>
@@ -16225,78 +16183,78 @@
       </c>
       <c r="G391" s="21"/>
     </row>
+    <row r="392" spans="1:7">
+      <c r="A392" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B392" s="54">
+        <v>350000597850</v>
+      </c>
+      <c r="C392" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="D392" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E392" s="57">
+        <v>1</v>
+      </c>
+      <c r="F392" s="58" t="s">
+        <v>12</v>
+      </c>
+      <c r="G392" s="21" t="s">
+        <v>170</v>
+      </c>
+    </row>
     <row r="393" spans="1:7">
-      <c r="A393" s="7" t="s">
+      <c r="A393" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B393" s="54">
+        <v>350000597852</v>
+      </c>
+      <c r="C393" s="55" t="s">
+        <v>171</v>
+      </c>
+      <c r="D393" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E393" s="57">
+        <v>1</v>
+      </c>
+      <c r="F393" s="58" t="s">
+        <v>12</v>
+      </c>
+      <c r="G393" s="21" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="395" spans="1:7">
+      <c r="A395" s="7" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="394" spans="1:7">
-      <c r="A394" s="43" t="s">
+    <row r="396" spans="1:7">
+      <c r="A396" s="43" t="s">
         <v>158</v>
       </c>
-      <c r="B394" s="44" t="s">
+      <c r="B396" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="C394" s="44" t="s">
+      <c r="C396" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="D394" s="45" t="s">
+      <c r="D396" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E394" s="44" t="s">
+      <c r="E396" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="F394" s="44" t="s">
+      <c r="F396" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="G394" s="44" t="s">
+      <c r="G396" s="44" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="395" spans="1:7">
-      <c r="A395" s="46" t="s">
-        <v>159</v>
-      </c>
-      <c r="B395" s="47">
-        <v>350001000403</v>
-      </c>
-      <c r="C395" s="46" t="s">
-        <v>160</v>
-      </c>
-      <c r="D395" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="E395" s="49">
-        <v>1</v>
-      </c>
-      <c r="F395" s="50" t="s">
-        <v>77</v>
-      </c>
-      <c r="G395" s="51" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="396" spans="1:7">
-      <c r="A396" s="46" t="s">
-        <v>159</v>
-      </c>
-      <c r="B396" s="47">
-        <v>350001042321</v>
-      </c>
-      <c r="C396" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D396" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="E396" s="49">
-        <v>1</v>
-      </c>
-      <c r="F396" s="50" t="s">
-        <v>77</v>
-      </c>
-      <c r="G396" s="51" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="397" spans="1:7">
@@ -16304,10 +16262,10 @@
         <v>159</v>
       </c>
       <c r="B397" s="47">
-        <v>350001042322</v>
+        <v>350001000403</v>
       </c>
       <c r="C397" s="46" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D397" s="48" t="s">
         <v>19</v>
@@ -16318,19 +16276,19 @@
       <c r="F397" s="50" t="s">
         <v>77</v>
       </c>
-      <c r="G397" s="50" t="s">
-        <v>164</v>
+      <c r="G397" s="51" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="398" spans="1:7">
       <c r="A398" s="46" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B398" s="47">
-        <v>350000592793</v>
+        <v>350001042321</v>
       </c>
       <c r="C398" s="46" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D398" s="48" t="s">
         <v>19</v>
@@ -16339,1675 +16297,99 @@
         <v>1</v>
       </c>
       <c r="F398" s="50" t="s">
-        <v>27</v>
-      </c>
-      <c r="G398" s="50"/>
+        <v>77</v>
+      </c>
+      <c r="G398" s="51" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="399" spans="1:7">
       <c r="A399" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="B399" s="47">
+        <v>350001042322</v>
+      </c>
+      <c r="C399" s="46" t="s">
+        <v>163</v>
+      </c>
+      <c r="D399" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="E399" s="49">
+        <v>1</v>
+      </c>
+      <c r="F399" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="G399" s="50" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="400" spans="1:7">
+      <c r="A400" s="46" t="s">
         <v>165</v>
       </c>
-      <c r="B399" s="47">
+      <c r="B400" s="47">
+        <v>350000592793</v>
+      </c>
+      <c r="C400" s="46" t="s">
+        <v>166</v>
+      </c>
+      <c r="D400" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="E400" s="49">
+        <v>1</v>
+      </c>
+      <c r="F400" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="G400" s="50"/>
+    </row>
+    <row r="401" spans="1:7">
+      <c r="A401" s="46" t="s">
+        <v>165</v>
+      </c>
+      <c r="B401" s="47">
         <v>350000592794</v>
       </c>
-      <c r="C399" s="46" t="s">
+      <c r="C401" s="46" t="s">
         <v>167</v>
       </c>
-      <c r="D399" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="E399" s="49">
-        <v>1</v>
-      </c>
-      <c r="F399" s="50" t="s">
+      <c r="D401" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="E401" s="49">
+        <v>1</v>
+      </c>
+      <c r="F401" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="G399" s="50"/>
-    </row>
-    <row r="400" spans="1:7">
-      <c r="A400" s="52"/>
-      <c r="B400" s="16"/>
-      <c r="C400" s="9"/>
-      <c r="D400" s="12"/>
-      <c r="E400" s="24"/>
-      <c r="F400" s="14"/>
-      <c r="G400" s="53"/>
-    </row>
-    <row r="401" spans="1:8">
-      <c r="A401" s="7" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="402" spans="1:8">
-      <c r="A402" t="s">
-        <v>170</v>
-      </c>
-      <c r="B402" t="s">
-        <v>2</v>
-      </c>
-      <c r="C402" t="s">
-        <v>3</v>
-      </c>
-      <c r="D402" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E402" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="F402" t="s">
-        <v>6</v>
-      </c>
-      <c r="G402" t="s">
-        <v>7</v>
-      </c>
-      <c r="H402" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="403" spans="1:8">
-      <c r="A403" t="s">
-        <v>172</v>
-      </c>
-      <c r="B403">
-        <v>350000597850</v>
-      </c>
-      <c r="C403" t="s">
-        <v>173</v>
-      </c>
-      <c r="D403" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E403" s="5">
-        <v>1</v>
-      </c>
-      <c r="F403" t="s">
-        <v>12</v>
-      </c>
-      <c r="G403" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="404" spans="1:8">
-      <c r="A404" t="s">
-        <v>172</v>
-      </c>
-      <c r="B404">
-        <v>350000597852</v>
-      </c>
-      <c r="C404" t="s">
-        <v>175</v>
-      </c>
-      <c r="D404" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E404" s="5">
-        <v>1</v>
-      </c>
-      <c r="F404" t="s">
-        <v>12</v>
-      </c>
-      <c r="G404" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="405" spans="1:8">
-      <c r="A405" t="s">
-        <v>177</v>
-      </c>
-      <c r="B405">
-        <v>350000589232</v>
-      </c>
-      <c r="C405" t="s">
-        <v>81</v>
-      </c>
-      <c r="D405" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E405" s="5">
-        <v>1</v>
-      </c>
-      <c r="F405" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="406" spans="1:8">
-      <c r="A406" t="s">
-        <v>177</v>
-      </c>
-      <c r="B406">
-        <v>350000589241</v>
-      </c>
-      <c r="C406" t="s">
-        <v>84</v>
-      </c>
-      <c r="D406" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E406" s="5">
-        <v>1</v>
-      </c>
-      <c r="F406" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="407" spans="1:8">
-      <c r="A407" t="s">
-        <v>177</v>
-      </c>
-      <c r="B407">
-        <v>350000589242</v>
-      </c>
-      <c r="C407" t="s">
-        <v>85</v>
-      </c>
-      <c r="D407" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E407" s="5">
-        <v>1</v>
-      </c>
-      <c r="F407" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="408" spans="1:8">
-      <c r="A408" t="s">
-        <v>177</v>
-      </c>
-      <c r="B408">
-        <v>350000589243</v>
-      </c>
-      <c r="C408" t="s">
-        <v>86</v>
-      </c>
-      <c r="D408" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E408" s="5">
-        <v>1</v>
-      </c>
-      <c r="F408" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="409" spans="1:8">
-      <c r="A409" t="s">
-        <v>177</v>
-      </c>
-      <c r="B409">
-        <v>350000589244</v>
-      </c>
-      <c r="C409" t="s">
-        <v>87</v>
-      </c>
-      <c r="D409" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E409" s="5">
-        <v>1</v>
-      </c>
-      <c r="F409" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="410" spans="1:8">
-      <c r="A410" t="s">
-        <v>177</v>
-      </c>
-      <c r="B410">
-        <v>350000589253</v>
-      </c>
-      <c r="C410" t="s">
-        <v>88</v>
-      </c>
-      <c r="D410" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E410" s="5">
-        <v>1</v>
-      </c>
-      <c r="F410" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="411" spans="1:8">
-      <c r="A411" t="s">
-        <v>177</v>
-      </c>
-      <c r="B411">
-        <v>350000589254</v>
-      </c>
-      <c r="C411" t="s">
-        <v>89</v>
-      </c>
-      <c r="D411" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E411" s="5">
-        <v>1</v>
-      </c>
-      <c r="F411" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="412" spans="1:8">
-      <c r="A412" t="s">
-        <v>177</v>
-      </c>
-      <c r="B412">
-        <v>350000589255</v>
-      </c>
-      <c r="C412" t="s">
-        <v>90</v>
-      </c>
-      <c r="D412" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E412" s="5">
-        <v>1</v>
-      </c>
-      <c r="F412" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="413" spans="1:8">
-      <c r="A413" t="s">
-        <v>177</v>
-      </c>
-      <c r="B413">
-        <v>350000589256</v>
-      </c>
-      <c r="C413" t="s">
-        <v>91</v>
-      </c>
-      <c r="D413" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E413" s="5">
-        <v>1</v>
-      </c>
-      <c r="F413" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="414" spans="1:8">
-      <c r="A414" t="s">
-        <v>177</v>
-      </c>
-      <c r="B414">
-        <v>350000589263</v>
-      </c>
-      <c r="C414" t="s">
-        <v>92</v>
-      </c>
-      <c r="D414" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E414" s="5">
-        <v>1</v>
-      </c>
-      <c r="F414" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="415" spans="1:8">
-      <c r="A415" t="s">
-        <v>177</v>
-      </c>
-      <c r="B415">
-        <v>350000589264</v>
-      </c>
-      <c r="C415" t="s">
-        <v>93</v>
-      </c>
-      <c r="D415" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E415" s="5">
-        <v>1</v>
-      </c>
-      <c r="F415" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="416" spans="1:8">
-      <c r="A416" t="s">
-        <v>177</v>
-      </c>
-      <c r="B416">
-        <v>350000589265</v>
-      </c>
-      <c r="C416" t="s">
-        <v>94</v>
-      </c>
-      <c r="D416" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E416" s="5">
-        <v>1</v>
-      </c>
-      <c r="F416" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="417" spans="1:6">
-      <c r="A417" t="s">
-        <v>177</v>
-      </c>
-      <c r="B417">
-        <v>350000589272</v>
-      </c>
-      <c r="C417" t="s">
-        <v>95</v>
-      </c>
-      <c r="D417" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E417" s="5">
-        <v>1</v>
-      </c>
-      <c r="F417" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="418" spans="1:6">
-      <c r="A418" t="s">
-        <v>177</v>
-      </c>
-      <c r="B418">
-        <v>350000589273</v>
-      </c>
-      <c r="C418" t="s">
-        <v>96</v>
-      </c>
-      <c r="D418" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E418" s="5">
-        <v>1</v>
-      </c>
-      <c r="F418" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="419" spans="1:6">
-      <c r="A419" t="s">
-        <v>177</v>
-      </c>
-      <c r="B419">
-        <v>350000589274</v>
-      </c>
-      <c r="C419" t="s">
-        <v>97</v>
-      </c>
-      <c r="D419" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E419" s="5">
-        <v>1</v>
-      </c>
-      <c r="F419" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="420" spans="1:6">
-      <c r="A420" t="s">
-        <v>177</v>
-      </c>
-      <c r="B420">
-        <v>350000589281</v>
-      </c>
-      <c r="C420" t="s">
-        <v>98</v>
-      </c>
-      <c r="D420" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E420" s="5">
-        <v>1</v>
-      </c>
-      <c r="F420" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="421" spans="1:6">
-      <c r="A421" t="s">
-        <v>177</v>
-      </c>
-      <c r="B421">
-        <v>350000589282</v>
-      </c>
-      <c r="C421" t="s">
-        <v>99</v>
-      </c>
-      <c r="D421" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E421" s="5">
-        <v>1</v>
-      </c>
-      <c r="F421" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="422" spans="1:6">
-      <c r="A422" t="s">
-        <v>177</v>
-      </c>
-      <c r="B422">
-        <v>350000589283</v>
-      </c>
-      <c r="C422" t="s">
-        <v>100</v>
-      </c>
-      <c r="D422" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E422" s="5">
-        <v>1</v>
-      </c>
-      <c r="F422" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="423" spans="1:6">
-      <c r="A423" t="s">
-        <v>177</v>
-      </c>
-      <c r="B423">
-        <v>350000589306</v>
-      </c>
-      <c r="C423" t="s">
-        <v>101</v>
-      </c>
-      <c r="D423" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E423" s="5">
-        <v>1</v>
-      </c>
-      <c r="F423" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="424" spans="1:6">
-      <c r="A424" t="s">
-        <v>177</v>
-      </c>
-      <c r="B424">
-        <v>350000589307</v>
-      </c>
-      <c r="C424" t="s">
-        <v>102</v>
-      </c>
-      <c r="D424" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E424" s="5">
-        <v>1</v>
-      </c>
-      <c r="F424" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="425" spans="1:6">
-      <c r="A425" t="s">
-        <v>177</v>
-      </c>
-      <c r="B425">
-        <v>350000589308</v>
-      </c>
-      <c r="C425" t="s">
-        <v>103</v>
-      </c>
-      <c r="D425" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E425" s="5">
-        <v>1</v>
-      </c>
-      <c r="F425" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="426" spans="1:6">
-      <c r="A426" t="s">
-        <v>177</v>
-      </c>
-      <c r="B426">
-        <v>350000589309</v>
-      </c>
-      <c r="C426" t="s">
-        <v>104</v>
-      </c>
-      <c r="D426" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E426" s="5">
-        <v>1</v>
-      </c>
-      <c r="F426" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="427" spans="1:6">
-      <c r="A427" t="s">
-        <v>177</v>
-      </c>
-      <c r="B427">
-        <v>350000589310</v>
-      </c>
-      <c r="C427" t="s">
-        <v>105</v>
-      </c>
-      <c r="D427" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E427" s="5">
-        <v>1</v>
-      </c>
-      <c r="F427" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="428" spans="1:6">
-      <c r="A428" t="s">
-        <v>177</v>
-      </c>
-      <c r="B428">
-        <v>350000589311</v>
-      </c>
-      <c r="C428" t="s">
-        <v>106</v>
-      </c>
-      <c r="D428" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E428" s="5">
-        <v>1</v>
-      </c>
-      <c r="F428" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="429" spans="1:6">
-      <c r="A429" t="s">
-        <v>177</v>
-      </c>
-      <c r="B429">
-        <v>350000589312</v>
-      </c>
-      <c r="C429" t="s">
-        <v>107</v>
-      </c>
-      <c r="D429" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E429" s="5">
-        <v>1</v>
-      </c>
-      <c r="F429" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="430" spans="1:6">
-      <c r="A430" t="s">
-        <v>177</v>
-      </c>
-      <c r="B430">
-        <v>350000589313</v>
-      </c>
-      <c r="C430" t="s">
-        <v>108</v>
-      </c>
-      <c r="D430" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E430" s="5">
-        <v>1</v>
-      </c>
-      <c r="F430" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="431" spans="1:6">
-      <c r="A431" t="s">
-        <v>177</v>
-      </c>
-      <c r="B431">
-        <v>350000589314</v>
-      </c>
-      <c r="C431" t="s">
-        <v>109</v>
-      </c>
-      <c r="D431" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E431" s="5">
-        <v>1</v>
-      </c>
-      <c r="F431" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="432" spans="1:6">
-      <c r="A432" t="s">
-        <v>177</v>
-      </c>
-      <c r="B432">
-        <v>350000589315</v>
-      </c>
-      <c r="C432" t="s">
-        <v>110</v>
-      </c>
-      <c r="D432" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E432" s="5">
-        <v>1</v>
-      </c>
-      <c r="F432" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="433" spans="1:8">
-      <c r="A433" t="s">
-        <v>177</v>
-      </c>
-      <c r="B433">
-        <v>350000589316</v>
-      </c>
-      <c r="C433" t="s">
-        <v>111</v>
-      </c>
-      <c r="D433" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E433" s="5">
-        <v>1</v>
-      </c>
-      <c r="F433" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="434" spans="1:8">
-      <c r="A434" t="s">
-        <v>177</v>
-      </c>
-      <c r="B434">
-        <v>350001095413</v>
-      </c>
-      <c r="C434" t="s">
-        <v>153</v>
-      </c>
-      <c r="D434" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E434" s="5">
-        <v>1</v>
-      </c>
-      <c r="F434" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="435" spans="1:8">
-      <c r="A435" t="s">
-        <v>177</v>
-      </c>
-      <c r="B435">
-        <v>350001095414</v>
-      </c>
-      <c r="C435" t="s">
-        <v>154</v>
-      </c>
-      <c r="D435" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E435" s="5">
-        <v>1</v>
-      </c>
-      <c r="F435" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="436" spans="1:8">
-      <c r="A436" t="s">
-        <v>177</v>
-      </c>
-      <c r="B436">
-        <v>350001095415</v>
-      </c>
-      <c r="C436" t="s">
-        <v>155</v>
-      </c>
-      <c r="D436" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E436" s="5">
-        <v>1</v>
-      </c>
-      <c r="F436" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="437" spans="1:8">
-      <c r="A437" t="s">
-        <v>177</v>
-      </c>
-      <c r="B437">
-        <v>350001095416</v>
-      </c>
-      <c r="C437" t="s">
-        <v>156</v>
-      </c>
-      <c r="D437" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E437" s="5">
-        <v>1</v>
-      </c>
-      <c r="F437" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="438" spans="1:8">
-      <c r="A438" t="s">
-        <v>178</v>
-      </c>
-      <c r="B438">
-        <v>350000214911</v>
-      </c>
-      <c r="C438" t="s">
-        <v>46</v>
-      </c>
-      <c r="D438" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E438" s="5">
-        <v>1</v>
-      </c>
-      <c r="F438" t="s">
-        <v>47</v>
-      </c>
-      <c r="G438" t="s">
-        <v>179</v>
-      </c>
-      <c r="H438" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="439" spans="1:8">
-      <c r="A439" t="s">
-        <v>178</v>
-      </c>
-      <c r="B439">
-        <v>350000214920</v>
-      </c>
-      <c r="C439" t="s">
-        <v>48</v>
-      </c>
-      <c r="D439" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E439" s="5">
-        <v>1</v>
-      </c>
-      <c r="F439" t="s">
-        <v>47</v>
-      </c>
-      <c r="G439" t="s">
-        <v>179</v>
-      </c>
-      <c r="H439" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="440" spans="1:8">
-      <c r="A440" t="s">
-        <v>178</v>
-      </c>
-      <c r="B440">
-        <v>350000214921</v>
-      </c>
-      <c r="C440" t="s">
-        <v>49</v>
-      </c>
-      <c r="D440" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E440" s="5">
-        <v>1</v>
-      </c>
-      <c r="F440" t="s">
-        <v>47</v>
-      </c>
-      <c r="G440" t="s">
-        <v>179</v>
-      </c>
-      <c r="H440" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="441" spans="1:8">
-      <c r="A441" t="s">
-        <v>178</v>
-      </c>
-      <c r="B441">
-        <v>350000214922</v>
-      </c>
-      <c r="C441" t="s">
-        <v>50</v>
-      </c>
-      <c r="D441" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E441" s="5">
-        <v>1</v>
-      </c>
-      <c r="F441" t="s">
-        <v>47</v>
-      </c>
-      <c r="G441" t="s">
-        <v>179</v>
-      </c>
-      <c r="H441" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="442" spans="1:8">
-      <c r="A442" t="s">
-        <v>178</v>
-      </c>
-      <c r="B442">
-        <v>350000214923</v>
-      </c>
-      <c r="C442" t="s">
-        <v>51</v>
-      </c>
-      <c r="D442" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E442" s="5">
-        <v>1</v>
-      </c>
-      <c r="F442" t="s">
-        <v>47</v>
-      </c>
-      <c r="G442" t="s">
-        <v>179</v>
-      </c>
-      <c r="H442" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="443" spans="1:8">
-      <c r="A443" t="s">
-        <v>178</v>
-      </c>
-      <c r="B443">
-        <v>350000475874</v>
-      </c>
-      <c r="C443" t="s">
-        <v>52</v>
-      </c>
-      <c r="D443" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E443" s="5">
-        <v>1</v>
-      </c>
-      <c r="F443" t="s">
-        <v>47</v>
-      </c>
-      <c r="G443" t="s">
-        <v>179</v>
-      </c>
-      <c r="H443" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="444" spans="1:8">
-      <c r="A444" t="s">
-        <v>178</v>
-      </c>
-      <c r="B444">
-        <v>350000475875</v>
-      </c>
-      <c r="C444" t="s">
-        <v>53</v>
-      </c>
-      <c r="D444" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E444" s="5">
-        <v>1</v>
-      </c>
-      <c r="F444" t="s">
-        <v>47</v>
-      </c>
-      <c r="G444" t="s">
-        <v>179</v>
-      </c>
-      <c r="H444" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="445" spans="1:8">
-      <c r="A445" t="s">
-        <v>178</v>
-      </c>
-      <c r="B445">
-        <v>350000475876</v>
-      </c>
-      <c r="C445" t="s">
-        <v>54</v>
-      </c>
-      <c r="D445" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E445" s="5">
-        <v>1</v>
-      </c>
-      <c r="F445" t="s">
-        <v>47</v>
-      </c>
-      <c r="G445" t="s">
-        <v>179</v>
-      </c>
-      <c r="H445" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="446" spans="1:8">
-      <c r="A446" t="s">
-        <v>178</v>
-      </c>
-      <c r="B446">
-        <v>350000475877</v>
-      </c>
-      <c r="C446" t="s">
-        <v>55</v>
-      </c>
-      <c r="D446" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E446" s="5">
-        <v>1</v>
-      </c>
-      <c r="F446" t="s">
-        <v>47</v>
-      </c>
-      <c r="G446" t="s">
-        <v>179</v>
-      </c>
-      <c r="H446" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="447" spans="1:8">
-      <c r="A447" t="s">
-        <v>178</v>
-      </c>
-      <c r="B447">
-        <v>350000214930</v>
-      </c>
-      <c r="C447" t="s">
-        <v>56</v>
-      </c>
-      <c r="D447" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E447" s="5">
-        <v>1</v>
-      </c>
-      <c r="F447" t="s">
-        <v>47</v>
-      </c>
-      <c r="G447" t="s">
-        <v>179</v>
-      </c>
-      <c r="H447" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="448" spans="1:8">
-      <c r="A448" t="s">
-        <v>178</v>
-      </c>
-      <c r="B448">
-        <v>350000214931</v>
-      </c>
-      <c r="C448" t="s">
-        <v>57</v>
-      </c>
-      <c r="D448" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E448" s="5">
-        <v>1</v>
-      </c>
-      <c r="F448" t="s">
-        <v>47</v>
-      </c>
-      <c r="G448" t="s">
-        <v>179</v>
-      </c>
-      <c r="H448" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="449" spans="1:8">
-      <c r="A449" t="s">
-        <v>178</v>
-      </c>
-      <c r="B449">
-        <v>350000214932</v>
-      </c>
-      <c r="C449" t="s">
-        <v>58</v>
-      </c>
-      <c r="D449" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E449" s="5">
-        <v>1</v>
-      </c>
-      <c r="F449" t="s">
-        <v>47</v>
-      </c>
-      <c r="G449" t="s">
-        <v>179</v>
-      </c>
-      <c r="H449" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="450" spans="1:8">
-      <c r="A450" t="s">
-        <v>178</v>
-      </c>
-      <c r="B450">
-        <v>350000214939</v>
-      </c>
-      <c r="C450" t="s">
-        <v>59</v>
-      </c>
-      <c r="D450" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E450" s="5">
-        <v>1</v>
-      </c>
-      <c r="F450" t="s">
-        <v>47</v>
-      </c>
-      <c r="G450" t="s">
-        <v>179</v>
-      </c>
-      <c r="H450" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="451" spans="1:8">
-      <c r="A451" t="s">
-        <v>178</v>
-      </c>
-      <c r="B451">
-        <v>350000214940</v>
-      </c>
-      <c r="C451" t="s">
-        <v>60</v>
-      </c>
-      <c r="D451" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E451" s="5">
-        <v>1</v>
-      </c>
-      <c r="F451" t="s">
-        <v>47</v>
-      </c>
-      <c r="G451" t="s">
-        <v>179</v>
-      </c>
-      <c r="H451" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="452" spans="1:8">
-      <c r="A452" t="s">
-        <v>178</v>
-      </c>
-      <c r="B452">
-        <v>350000214941</v>
-      </c>
-      <c r="C452" t="s">
-        <v>61</v>
-      </c>
-      <c r="D452" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E452" s="5">
-        <v>1</v>
-      </c>
-      <c r="F452" t="s">
-        <v>47</v>
-      </c>
-      <c r="G452" t="s">
-        <v>179</v>
-      </c>
-      <c r="H452" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="453" spans="1:8">
-      <c r="A453" t="s">
-        <v>178</v>
-      </c>
-      <c r="B453">
-        <v>350000298408</v>
-      </c>
-      <c r="C453" t="s">
-        <v>62</v>
-      </c>
-      <c r="D453" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E453" s="5">
-        <v>1</v>
-      </c>
-      <c r="F453" t="s">
-        <v>47</v>
-      </c>
-      <c r="G453" t="s">
-        <v>179</v>
-      </c>
-      <c r="H453" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="454" spans="1:8">
-      <c r="A454" t="s">
-        <v>178</v>
-      </c>
-      <c r="B454">
-        <v>350000298409</v>
-      </c>
-      <c r="C454" t="s">
-        <v>63</v>
-      </c>
-      <c r="D454" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E454" s="5">
-        <v>1</v>
-      </c>
-      <c r="F454" t="s">
-        <v>47</v>
-      </c>
-      <c r="G454" t="s">
-        <v>179</v>
-      </c>
-      <c r="H454" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="455" spans="1:8">
-      <c r="A455" t="s">
-        <v>178</v>
-      </c>
-      <c r="B455">
-        <v>350000298410</v>
-      </c>
-      <c r="C455" t="s">
-        <v>64</v>
-      </c>
-      <c r="D455" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E455" s="5">
-        <v>1</v>
-      </c>
-      <c r="F455" t="s">
-        <v>47</v>
-      </c>
-      <c r="G455" t="s">
-        <v>179</v>
-      </c>
-      <c r="H455" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="456" spans="1:8">
-      <c r="A456" t="s">
-        <v>178</v>
-      </c>
-      <c r="B456">
-        <v>350000212468</v>
-      </c>
-      <c r="C456" t="s">
-        <v>65</v>
-      </c>
-      <c r="D456" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E456" s="5">
-        <v>1</v>
-      </c>
-      <c r="F456" t="s">
-        <v>47</v>
-      </c>
-      <c r="G456" t="s">
-        <v>179</v>
-      </c>
-      <c r="H456" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="457" spans="1:8">
-      <c r="A457" t="s">
-        <v>178</v>
-      </c>
-      <c r="B457">
-        <v>350000212469</v>
-      </c>
-      <c r="C457" t="s">
-        <v>66</v>
-      </c>
-      <c r="D457" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E457" s="5">
-        <v>1</v>
-      </c>
-      <c r="F457" t="s">
-        <v>47</v>
-      </c>
-      <c r="G457" t="s">
-        <v>179</v>
-      </c>
-      <c r="H457" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="458" spans="1:8">
-      <c r="A458" t="s">
-        <v>178</v>
-      </c>
-      <c r="B458">
-        <v>350000212470</v>
-      </c>
-      <c r="C458" t="s">
-        <v>67</v>
-      </c>
-      <c r="D458" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E458" s="5">
-        <v>1</v>
-      </c>
-      <c r="F458" t="s">
-        <v>47</v>
-      </c>
-      <c r="G458" t="s">
-        <v>179</v>
-      </c>
-      <c r="H458" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="459" spans="1:8">
-      <c r="A459" t="s">
-        <v>178</v>
-      </c>
-      <c r="B459">
-        <v>350000212471</v>
-      </c>
-      <c r="C459" t="s">
-        <v>68</v>
-      </c>
-      <c r="D459" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E459" s="5">
-        <v>1</v>
-      </c>
-      <c r="F459" t="s">
-        <v>47</v>
-      </c>
-      <c r="G459" t="s">
-        <v>179</v>
-      </c>
-      <c r="H459" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="460" spans="1:8">
-      <c r="A460" t="s">
-        <v>178</v>
-      </c>
-      <c r="B460">
-        <v>350000212472</v>
-      </c>
-      <c r="C460" t="s">
-        <v>69</v>
-      </c>
-      <c r="D460" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E460" s="5">
-        <v>1</v>
-      </c>
-      <c r="F460" t="s">
-        <v>47</v>
-      </c>
-      <c r="G460" t="s">
-        <v>179</v>
-      </c>
-      <c r="H460" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="461" spans="1:8">
-      <c r="A461" t="s">
-        <v>178</v>
-      </c>
-      <c r="B461">
-        <v>350000212473</v>
-      </c>
-      <c r="C461" t="s">
-        <v>70</v>
-      </c>
-      <c r="D461" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E461" s="5">
-        <v>1</v>
-      </c>
-      <c r="F461" t="s">
-        <v>47</v>
-      </c>
-      <c r="G461" t="s">
-        <v>179</v>
-      </c>
-      <c r="H461" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="462" spans="1:8">
-      <c r="A462" t="s">
-        <v>178</v>
-      </c>
-      <c r="B462">
-        <v>350000358611</v>
-      </c>
-      <c r="C462" t="s">
-        <v>71</v>
-      </c>
-      <c r="D462" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E462" s="5">
-        <v>1</v>
-      </c>
-      <c r="F462" t="s">
-        <v>47</v>
-      </c>
-      <c r="G462" t="s">
-        <v>179</v>
-      </c>
-      <c r="H462" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="463" spans="1:8">
-      <c r="A463" t="s">
-        <v>178</v>
-      </c>
-      <c r="B463">
-        <v>350000212474</v>
-      </c>
-      <c r="C463" t="s">
-        <v>72</v>
-      </c>
-      <c r="D463" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E463" s="5">
-        <v>1</v>
-      </c>
-      <c r="F463" t="s">
-        <v>47</v>
-      </c>
-      <c r="G463" t="s">
-        <v>179</v>
-      </c>
-      <c r="H463" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="464" spans="1:8">
-      <c r="A464" t="s">
-        <v>178</v>
-      </c>
-      <c r="B464">
-        <v>350000212475</v>
-      </c>
-      <c r="C464" t="s">
-        <v>73</v>
-      </c>
-      <c r="D464" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E464" s="5">
-        <v>1</v>
-      </c>
-      <c r="F464" t="s">
-        <v>47</v>
-      </c>
-      <c r="G464" t="s">
-        <v>179</v>
-      </c>
-      <c r="H464" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="465" spans="1:8">
-      <c r="A465" t="s">
-        <v>178</v>
-      </c>
-      <c r="B465">
-        <v>350000212476</v>
-      </c>
-      <c r="C465" t="s">
-        <v>74</v>
-      </c>
-      <c r="D465" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E465" s="5">
-        <v>1</v>
-      </c>
-      <c r="F465" t="s">
-        <v>47</v>
-      </c>
-      <c r="G465" t="s">
-        <v>179</v>
-      </c>
-      <c r="H465" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="466" spans="1:8">
-      <c r="A466" t="s">
-        <v>178</v>
-      </c>
-      <c r="B466">
-        <v>350000589206</v>
-      </c>
-      <c r="C466" t="s">
-        <v>75</v>
-      </c>
-      <c r="D466" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E466" s="5">
-        <v>1</v>
-      </c>
-      <c r="F466" t="s">
-        <v>47</v>
-      </c>
-      <c r="G466" t="s">
-        <v>179</v>
-      </c>
-      <c r="H466" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="467" spans="1:8">
-      <c r="A467" t="s">
-        <v>178</v>
-      </c>
-      <c r="B467">
-        <v>350001095409</v>
-      </c>
-      <c r="C467" t="s">
-        <v>132</v>
-      </c>
-      <c r="D467" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E467" s="5">
-        <v>1</v>
-      </c>
-      <c r="F467" t="s">
-        <v>133</v>
-      </c>
-      <c r="G467" t="s">
-        <v>179</v>
-      </c>
-      <c r="H467" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="468" spans="1:8">
-      <c r="A468" t="s">
-        <v>178</v>
-      </c>
-      <c r="B468">
-        <v>350001095410</v>
-      </c>
-      <c r="C468" t="s">
-        <v>134</v>
-      </c>
-      <c r="D468" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E468" s="5">
-        <v>1</v>
-      </c>
-      <c r="F468" t="s">
-        <v>133</v>
-      </c>
-      <c r="G468" t="s">
-        <v>179</v>
-      </c>
-      <c r="H468" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="469" spans="1:8">
-      <c r="A469" t="s">
-        <v>178</v>
-      </c>
-      <c r="B469">
-        <v>350001095411</v>
-      </c>
-      <c r="C469" t="s">
-        <v>135</v>
-      </c>
-      <c r="D469" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E469" s="5">
-        <v>1</v>
-      </c>
-      <c r="F469" t="s">
-        <v>133</v>
-      </c>
-      <c r="G469" t="s">
-        <v>179</v>
-      </c>
-      <c r="H469" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="470" spans="1:8">
-      <c r="A470" t="s">
-        <v>178</v>
-      </c>
-      <c r="B470">
-        <v>350001095412</v>
-      </c>
-      <c r="C470" t="s">
-        <v>136</v>
-      </c>
-      <c r="D470" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E470" s="5">
-        <v>1</v>
-      </c>
-      <c r="F470" t="s">
-        <v>133</v>
-      </c>
-      <c r="G470" t="s">
-        <v>179</v>
-      </c>
-      <c r="H470" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="471" spans="1:8">
-      <c r="A471" t="s">
-        <v>181</v>
-      </c>
-      <c r="B471">
-        <v>350000499960</v>
-      </c>
-      <c r="C471" t="s">
-        <v>182</v>
-      </c>
-      <c r="D471" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="E471" s="5">
-        <v>1</v>
-      </c>
-      <c r="F471" t="s">
-        <v>12</v>
-      </c>
-      <c r="G471" t="s">
-        <v>184</v>
-      </c>
-      <c r="H471" t="s">
-        <v>180</v>
-      </c>
+      <c r="G401" s="50"/>
+    </row>
+    <row r="402" spans="1:7">
+      <c r="A402" s="52"/>
+      <c r="B402" s="16"/>
+      <c r="C402" s="9"/>
+      <c r="D402" s="12"/>
+      <c r="E402" s="24"/>
+      <c r="F402" s="14"/>
+      <c r="G402" s="53"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="37" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
-  <tableParts count="4">
+  <tableParts count="3">
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
-    <tablePart r:id="rId6"/>
   </tableParts>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{3A4CF648-6AED-40f4-86FF-DC5316D8AED3}">
       <x14:slicerList xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicer r:id="rId7"/>
+        <x14:slicer r:id="rId6"/>
       </x14:slicerList>
     </ext>
   </extLst>

</xml_diff>